<commit_message>
set prepared to merge 25 Msrch
</commit_message>
<xml_diff>
--- a/cost_final24.xlsx
+++ b/cost_final24.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\1_UPM_Z\PYsimul\SMR_model1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{857B72B2-D90F-42FA-A1ED-78702E95CDAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6264ABD4-21A2-4C1A-BCC1-D144512A6B48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38310" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1049,10 +1049,44 @@
       <c r="A13" s="2" t="s">
         <v>25</v>
       </c>
+      <c r="B13" s="3">
+        <v>3000</v>
+      </c>
+      <c r="C13" s="4">
+        <v>100</v>
+      </c>
+      <c r="D13" s="4">
+        <v>2</v>
+      </c>
       <c r="E13" s="4">
         <v>60</v>
       </c>
       <c r="F13" s="4">
+        <v>0</v>
+      </c>
+      <c r="G13" s="4">
+        <v>7</v>
+      </c>
+      <c r="H13" s="4">
+        <f>7.15</f>
+        <v>7.15</v>
+      </c>
+      <c r="I13" s="4">
+        <v>0</v>
+      </c>
+      <c r="J13" s="4">
+        <v>300</v>
+      </c>
+      <c r="K13" s="4">
+        <v>0.85</v>
+      </c>
+      <c r="L13" s="4">
+        <v>0.05</v>
+      </c>
+      <c r="M13" s="5">
+        <v>0</v>
+      </c>
+      <c r="N13" s="5">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
set costs 6 March
</commit_message>
<xml_diff>
--- a/cost_final24.xlsx
+++ b/cost_final24.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\1_UPM_Z\PYsimul\SMR_model1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6264ABD4-21A2-4C1A-BCC1-D144512A6B48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A0B3242-A4CF-4C7F-B5D1-6072480F42FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38310" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1094,6 +1094,46 @@
       <c r="A14" s="2" t="s">
         <v>26</v>
       </c>
+      <c r="B14" s="4">
+        <v>750</v>
+      </c>
+      <c r="C14" s="4">
+        <v>20.167538959821201</v>
+      </c>
+      <c r="D14" s="4">
+        <v>1.827</v>
+      </c>
+      <c r="E14" s="4">
+        <v>30</v>
+      </c>
+      <c r="F14" s="4">
+        <v>0.59</v>
+      </c>
+      <c r="G14" s="4">
+        <v>2</v>
+      </c>
+      <c r="H14" s="4">
+        <f>50</f>
+        <v>50</v>
+      </c>
+      <c r="I14" s="4">
+        <v>450</v>
+      </c>
+      <c r="J14" s="4">
+        <v>500</v>
+      </c>
+      <c r="K14" s="4">
+        <v>0.85</v>
+      </c>
+      <c r="L14" s="4">
+        <v>0.05</v>
+      </c>
+      <c r="M14" s="5">
+        <v>0</v>
+      </c>
+      <c r="N14" s="5">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
get costs SMR and energy breakdown
</commit_message>
<xml_diff>
--- a/cost_final24.xlsx
+++ b/cost_final24.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\1_UPM_Z\PYsimul\SMR_model1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A0B3242-A4CF-4C7F-B5D1-6072480F42FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D79C42FA-AE12-4C24-819C-685A2EC3B6FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,6 +35,33 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={D0289C43-A833-42EB-B6DD-035525C890A0}</author>
+    <author>tc={5E7A287D-12A6-4C51-8940-91185041EAD9}</author>
+  </authors>
+  <commentList>
+    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{D0289C43-A833-42EB-B6DD-035525C890A0}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Relativo al CO2</t>
+      </text>
+    </comment>
+    <comment ref="G14" authorId="1" shapeId="0" xr:uid="{5E7A287D-12A6-4C51-8940-91185041EAD9}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Buscar fuente para esto</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
@@ -123,7 +150,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -151,6 +178,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -209,6 +242,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="CARLOS OLMOS ALONSO" id="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" userId="S::carlos.olmos.alonso@alumnos.upm.es::b1989f31-5088-41d6-9a36-5ce09ab23a53" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -472,8 +511,19 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="F1" dT="2025-04-07T12:41:32.37" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{D0289C43-A833-42EB-B6DD-035525C890A0}">
+    <text>Relativo al CO2</text>
+  </threadedComment>
+  <threadedComment ref="G14" dT="2025-04-07T12:44:05.12" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{5E7A287D-12A6-4C51-8940-91185041EAD9}">
+    <text>Buscar fuente para esto</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -488,7 +538,7 @@
     <col min="9" max="9" width="17.6328125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.08984375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.6328125" customWidth="1"/>
     <col min="13" max="13" width="4.36328125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="13.08984375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="20" bestFit="1" customWidth="1"/>
@@ -1050,13 +1100,13 @@
         <v>25</v>
       </c>
       <c r="B13" s="3">
-        <v>3000</v>
+        <v>9500</v>
       </c>
       <c r="C13" s="4">
-        <v>100</v>
+        <v>216</v>
       </c>
       <c r="D13" s="4">
-        <v>2</v>
+        <v>2.8</v>
       </c>
       <c r="E13" s="4">
         <v>60</v>
@@ -1068,8 +1118,8 @@
         <v>7</v>
       </c>
       <c r="H13" s="4">
-        <f>7.15</f>
-        <v>7.15</v>
+        <f>12</f>
+        <v>12</v>
       </c>
       <c r="I13" s="4">
         <v>0</v>
@@ -1078,10 +1128,10 @@
         <v>300</v>
       </c>
       <c r="K13" s="4">
-        <v>0.85</v>
+        <v>0.93</v>
       </c>
       <c r="L13" s="4">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
       <c r="M13" s="5">
         <v>0</v>
@@ -1107,10 +1157,12 @@
         <v>30</v>
       </c>
       <c r="F14" s="4">
+        <f>0.59</f>
         <v>0.59</v>
       </c>
       <c r="G14" s="4">
-        <v>2</v>
+        <f>3</f>
+        <v>3</v>
       </c>
       <c r="H14" s="4">
         <f>50</f>
@@ -1138,5 +1190,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
set costs start market 15 April
</commit_message>
<xml_diff>
--- a/cost_final24.xlsx
+++ b/cost_final24.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\1_UPM_Z\PYsimul\SMR_model1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D79C42FA-AE12-4C24-819C-685A2EC3B6FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBBADF9B-E08B-4938-8959-DE6DB8AF3E45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,6 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={D0289C43-A833-42EB-B6DD-035525C890A0}</author>
-    <author>tc={5E7A287D-12A6-4C51-8940-91185041EAD9}</author>
   </authors>
   <commentList>
     <comment ref="F1" authorId="0" shapeId="0" xr:uid="{D0289C43-A833-42EB-B6DD-035525C890A0}">
@@ -48,14 +47,6 @@
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Relativo al CO2</t>
-      </text>
-    </comment>
-    <comment ref="G14" authorId="1" shapeId="0" xr:uid="{5E7A287D-12A6-4C51-8940-91185041EAD9}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Buscar fuente para esto</t>
       </text>
     </comment>
   </commentList>
@@ -180,26 +171,47 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4CCCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -220,12 +232,14 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -516,9 +530,6 @@
   <threadedComment ref="F1" dT="2025-04-07T12:41:32.37" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{D0289C43-A833-42EB-B6DD-035525C890A0}">
     <text>Relativo al CO2</text>
   </threadedComment>
-  <threadedComment ref="G14" dT="2025-04-07T12:44:05.12" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{5E7A287D-12A6-4C51-8940-91185041EAD9}">
-    <text>Buscar fuente para esto</text>
-  </threadedComment>
 </ThreadedComments>
 </file>
 
@@ -633,10 +644,10 @@
       <c r="L2" s="4">
         <v>0.05</v>
       </c>
-      <c r="M2" s="5">
-        <v>0</v>
-      </c>
-      <c r="N2" s="5">
+      <c r="M2" s="4">
+        <v>0</v>
+      </c>
+      <c r="N2" s="4">
         <v>0</v>
       </c>
     </row>
@@ -677,10 +688,10 @@
       <c r="L3" s="4">
         <v>0.05</v>
       </c>
-      <c r="M3" s="5">
-        <v>0</v>
-      </c>
-      <c r="N3" s="5">
+      <c r="M3" s="4">
+        <v>0</v>
+      </c>
+      <c r="N3" s="4">
         <v>0</v>
       </c>
     </row>
@@ -697,7 +708,7 @@
       <c r="D4" s="4">
         <v>0</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="5">
         <v>30</v>
       </c>
       <c r="F4" s="4">
@@ -712,19 +723,19 @@
       <c r="I4" s="4">
         <v>0</v>
       </c>
-      <c r="J4" s="7">
+      <c r="J4" s="4">
         <v>50</v>
       </c>
-      <c r="K4" s="7">
+      <c r="K4" s="4">
         <v>0.3</v>
       </c>
       <c r="L4" s="4">
         <v>0.05</v>
       </c>
-      <c r="M4" s="5">
-        <v>0</v>
-      </c>
-      <c r="N4" s="5">
+      <c r="M4" s="4">
+        <v>0</v>
+      </c>
+      <c r="N4" s="4">
         <v>0</v>
       </c>
     </row>
@@ -756,19 +767,19 @@
       <c r="I5" s="4">
         <v>0</v>
       </c>
-      <c r="J5" s="7">
+      <c r="J5" s="4">
         <v>50</v>
       </c>
-      <c r="K5" s="7">
+      <c r="K5" s="4">
         <v>0.2</v>
       </c>
       <c r="L5" s="4">
         <v>0.05</v>
       </c>
-      <c r="M5" s="5">
-        <v>0</v>
-      </c>
-      <c r="N5" s="5">
+      <c r="M5" s="4">
+        <v>0</v>
+      </c>
+      <c r="N5" s="4">
         <v>0</v>
       </c>
     </row>
@@ -810,10 +821,10 @@
       <c r="L6" s="4">
         <v>0.05</v>
       </c>
-      <c r="M6" s="5">
-        <v>0</v>
-      </c>
-      <c r="N6" s="5">
+      <c r="M6" s="4">
+        <v>0</v>
+      </c>
+      <c r="N6" s="4">
         <v>0</v>
       </c>
     </row>
@@ -854,10 +865,10 @@
       <c r="L7" s="4">
         <v>0.05</v>
       </c>
-      <c r="M7" s="5">
-        <v>0</v>
-      </c>
-      <c r="N7" s="5">
+      <c r="M7" s="4">
+        <v>0</v>
+      </c>
+      <c r="N7" s="4">
         <v>0</v>
       </c>
     </row>
@@ -898,10 +909,10 @@
       <c r="L8" s="4">
         <v>0.05</v>
       </c>
-      <c r="M8" s="5">
-        <v>0</v>
-      </c>
-      <c r="N8" s="5">
+      <c r="M8" s="4">
+        <v>0</v>
+      </c>
+      <c r="N8" s="4">
         <v>0</v>
       </c>
     </row>
@@ -918,7 +929,7 @@
       <c r="D9" s="4">
         <v>0</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="5">
         <v>60</v>
       </c>
       <c r="F9" s="4">
@@ -936,16 +947,16 @@
       <c r="J9" s="4">
         <v>500</v>
       </c>
-      <c r="K9" s="7">
+      <c r="K9" s="4">
         <v>0.2</v>
       </c>
       <c r="L9" s="4">
         <v>0.05</v>
       </c>
-      <c r="M9" s="5">
-        <v>0</v>
-      </c>
-      <c r="N9" s="5">
+      <c r="M9" s="4">
+        <v>0</v>
+      </c>
+      <c r="N9" s="4">
         <v>0</v>
       </c>
     </row>
@@ -980,17 +991,17 @@
       <c r="J10" s="4">
         <v>5</v>
       </c>
-      <c r="K10" s="7">
+      <c r="K10" s="4">
         <f>0.6</f>
         <v>0.6</v>
       </c>
       <c r="L10" s="4">
         <v>0.05</v>
       </c>
-      <c r="M10" s="5">
-        <v>0</v>
-      </c>
-      <c r="N10" s="5">
+      <c r="M10" s="4">
+        <v>0</v>
+      </c>
+      <c r="N10" s="4">
         <v>0</v>
       </c>
     </row>
@@ -1025,16 +1036,16 @@
       <c r="J11" s="4">
         <v>50</v>
       </c>
-      <c r="K11" s="7">
+      <c r="K11" s="4">
         <v>0.2</v>
       </c>
       <c r="L11" s="4">
         <v>0.05</v>
       </c>
-      <c r="M11" s="5">
-        <v>0</v>
-      </c>
-      <c r="N11" s="5">
+      <c r="M11" s="4">
+        <v>0</v>
+      </c>
+      <c r="N11" s="4">
         <v>0</v>
       </c>
     </row>
@@ -1078,7 +1089,7 @@
         <f>50</f>
         <v>50</v>
       </c>
-      <c r="K12" s="7">
+      <c r="K12" s="4">
         <f>0.4</f>
         <v>0.4</v>
       </c>
@@ -1086,16 +1097,16 @@
         <f>0.05</f>
         <v>0.05</v>
       </c>
-      <c r="M12" s="5">
+      <c r="M12" s="4">
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="N12" s="5">
+      <c r="N12" s="4">
         <f>0</f>
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="17" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:14" ht="17.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>25</v>
       </c>
@@ -1133,57 +1144,58 @@
       <c r="L13" s="4">
         <v>0.08</v>
       </c>
-      <c r="M13" s="5">
-        <v>0</v>
-      </c>
-      <c r="N13" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" ht="17" x14ac:dyDescent="0.35">
+      <c r="M13" s="4">
+        <v>0</v>
+      </c>
+      <c r="N13" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="17.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="4">
-        <v>750</v>
-      </c>
-      <c r="C14" s="4">
-        <v>20.167538959821201</v>
-      </c>
-      <c r="D14" s="4">
-        <v>1.827</v>
-      </c>
-      <c r="E14" s="4">
-        <v>30</v>
-      </c>
-      <c r="F14" s="4">
-        <f>0.59</f>
-        <v>0.59</v>
-      </c>
-      <c r="G14" s="4">
-        <f>3</f>
-        <v>3</v>
-      </c>
-      <c r="H14" s="4">
+      <c r="B14" s="6">
+        <f>583.13</f>
+        <v>583.13</v>
+      </c>
+      <c r="C14" s="6">
+        <v>20.63</v>
+      </c>
+      <c r="D14" s="7">
+        <v>5.5</v>
+      </c>
+      <c r="E14" s="6">
+        <v>25</v>
+      </c>
+      <c r="F14" s="6">
+        <v>0.41499999999999998</v>
+      </c>
+      <c r="G14" s="6">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="H14" s="6">
         <f>50</f>
         <v>50</v>
       </c>
-      <c r="I14" s="4">
+      <c r="I14" s="6">
+        <f>450</f>
         <v>450</v>
       </c>
-      <c r="J14" s="4">
-        <v>500</v>
-      </c>
-      <c r="K14" s="4">
+      <c r="J14" s="6">
+        <v>100</v>
+      </c>
+      <c r="K14" s="6">
         <v>0.85</v>
       </c>
-      <c r="L14" s="4">
+      <c r="L14" s="6">
         <v>0.05</v>
       </c>
-      <c r="M14" s="5">
-        <v>0</v>
-      </c>
-      <c r="N14" s="5">
+      <c r="M14" s="6">
+        <v>0</v>
+      </c>
+      <c r="N14" s="6">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
set Carbon cost to find threshold 11 May
</commit_message>
<xml_diff>
--- a/cost_final24.xlsx
+++ b/cost_final24.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\1_UPM_Z\PYsimul\SMR_model1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22129071-2FD4-41E0-9290-893ECE36F38D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B09C8DF-2CD6-4C81-9320-E0596127D6AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="38620" windowHeight="21820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>nuclear</t>
   </si>
@@ -135,6 +135,9 @@
   </si>
   <si>
     <t>Gas_CHP</t>
+  </si>
+  <si>
+    <t>carbon_intensity1</t>
   </si>
 </sst>
 </file>
@@ -535,7 +538,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.08984375" bestFit="1" customWidth="1"/>
@@ -547,23 +550,24 @@
     <col min="7" max="7" width="19.08984375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="5.36328125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.08984375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.6328125" customWidth="1"/>
-    <col min="13" max="13" width="4.36328125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.08984375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="20" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="16.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="24.26953125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="20" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.6328125" customWidth="1"/>
+    <col min="11" max="11" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.6328125" customWidth="1"/>
+    <col min="14" max="14" width="4.36328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.08984375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="24.26953125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="20" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="17" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" ht="17" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>23</v>
       </c>
@@ -592,22 +596,25 @@
         <v>13</v>
       </c>
       <c r="J1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="17" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" ht="17" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -636,22 +643,26 @@
         <v>0</v>
       </c>
       <c r="J2" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="K2" s="4">
         <v>1000</v>
       </c>
-      <c r="K2" s="4">
+      <c r="L2" s="4">
         <v>0.85</v>
       </c>
-      <c r="L2" s="4">
+      <c r="M2" s="4">
         <v>0.05</v>
       </c>
-      <c r="M2" s="4">
-        <v>0</v>
-      </c>
       <c r="N2" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" ht="17" x14ac:dyDescent="0.35">
+      <c r="O2" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" ht="17" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -680,22 +691,26 @@
         <v>0</v>
       </c>
       <c r="J3" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="K3" s="4">
         <v>1000</v>
       </c>
-      <c r="K3" s="4">
+      <c r="L3" s="4">
         <v>0.85</v>
       </c>
-      <c r="L3" s="4">
+      <c r="M3" s="4">
         <v>0.05</v>
       </c>
-      <c r="M3" s="4">
-        <v>0</v>
-      </c>
       <c r="N3" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" ht="17" x14ac:dyDescent="0.35">
+      <c r="O3" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="17" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -724,22 +739,26 @@
         <v>0</v>
       </c>
       <c r="J4" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="K4" s="4">
         <v>50</v>
       </c>
-      <c r="K4" s="4">
+      <c r="L4" s="4">
         <v>0.3</v>
       </c>
-      <c r="L4" s="4">
+      <c r="M4" s="4">
         <v>0.05</v>
       </c>
-      <c r="M4" s="4">
-        <v>0</v>
-      </c>
       <c r="N4" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" ht="17" x14ac:dyDescent="0.35">
+      <c r="O4" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="17" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -768,22 +787,26 @@
         <v>0</v>
       </c>
       <c r="J5" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="K5" s="4">
         <v>50</v>
       </c>
-      <c r="K5" s="4">
+      <c r="L5" s="4">
         <v>0.2</v>
       </c>
-      <c r="L5" s="4">
+      <c r="M5" s="4">
         <v>0.05</v>
       </c>
-      <c r="M5" s="4">
-        <v>0</v>
-      </c>
       <c r="N5" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" ht="17" x14ac:dyDescent="0.35">
+      <c r="O5" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="17" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -813,22 +836,26 @@
         <v>450</v>
       </c>
       <c r="J6" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="K6" s="4">
         <v>500</v>
       </c>
-      <c r="K6" s="4">
+      <c r="L6" s="4">
         <v>0.85</v>
       </c>
-      <c r="L6" s="4">
+      <c r="M6" s="4">
         <v>0.05</v>
       </c>
-      <c r="M6" s="4">
-        <v>0</v>
-      </c>
       <c r="N6" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" ht="17" x14ac:dyDescent="0.35">
+      <c r="O6" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" ht="17" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -857,22 +884,26 @@
         <v>850</v>
       </c>
       <c r="J7" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="K7" s="4">
         <v>500</v>
       </c>
-      <c r="K7" s="4">
+      <c r="L7" s="4">
         <v>0.85</v>
       </c>
-      <c r="L7" s="4">
+      <c r="M7" s="4">
         <v>0.05</v>
       </c>
-      <c r="M7" s="4">
-        <v>0</v>
-      </c>
       <c r="N7" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" ht="17" x14ac:dyDescent="0.35">
+      <c r="O7" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" ht="17" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -901,22 +932,26 @@
         <v>0</v>
       </c>
       <c r="J8" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="K8" s="4">
         <v>100</v>
       </c>
-      <c r="K8" s="4">
+      <c r="L8" s="4">
         <v>0.5</v>
       </c>
-      <c r="L8" s="4">
+      <c r="M8" s="4">
         <v>0.05</v>
       </c>
-      <c r="M8" s="4">
-        <v>0</v>
-      </c>
       <c r="N8" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" ht="17" x14ac:dyDescent="0.35">
+      <c r="O8" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" ht="17" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -945,22 +980,26 @@
         <v>0</v>
       </c>
       <c r="J9" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="K9" s="4">
         <v>500</v>
       </c>
-      <c r="K9" s="4">
+      <c r="L9" s="4">
         <v>0.2</v>
       </c>
-      <c r="L9" s="4">
+      <c r="M9" s="4">
         <v>0.05</v>
       </c>
-      <c r="M9" s="4">
-        <v>0</v>
-      </c>
       <c r="N9" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:14" ht="17" x14ac:dyDescent="0.35">
+      <c r="O9" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" ht="17" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -989,23 +1028,27 @@
         <v>0</v>
       </c>
       <c r="J10" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="K10" s="4">
         <v>5</v>
       </c>
-      <c r="K10" s="4">
+      <c r="L10" s="4">
         <f>0.6</f>
         <v>0.6</v>
       </c>
-      <c r="L10" s="4">
+      <c r="M10" s="4">
         <v>0.05</v>
       </c>
-      <c r="M10" s="4">
-        <v>0</v>
-      </c>
       <c r="N10" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:14" ht="17" x14ac:dyDescent="0.35">
+      <c r="O10" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" ht="17" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -1034,22 +1077,26 @@
         <v>0</v>
       </c>
       <c r="J11" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="K11" s="4">
         <v>50</v>
       </c>
-      <c r="K11" s="4">
+      <c r="L11" s="4">
         <v>0.2</v>
       </c>
-      <c r="L11" s="4">
+      <c r="M11" s="4">
         <v>0.05</v>
       </c>
-      <c r="M11" s="4">
-        <v>0</v>
-      </c>
       <c r="N11" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:14" ht="17" x14ac:dyDescent="0.35">
+      <c r="O11" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" ht="17" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>24</v>
       </c>
@@ -1086,27 +1133,31 @@
         <v>0</v>
       </c>
       <c r="J12" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="K12" s="4">
         <f>50</f>
         <v>50</v>
       </c>
-      <c r="K12" s="4">
+      <c r="L12" s="4">
         <f>0.4</f>
         <v>0.4</v>
       </c>
-      <c r="L12" s="4">
+      <c r="M12" s="4">
         <f>0.05</f>
         <v>0.05</v>
       </c>
-      <c r="M12" s="4">
-        <f>0</f>
-        <v>0</v>
-      </c>
       <c r="N12" s="4">
         <f>0</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:14" ht="17.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="O12" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" ht="17.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>25</v>
       </c>
@@ -1136,22 +1187,26 @@
         <v>0</v>
       </c>
       <c r="J13" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="K13" s="4">
         <v>300</v>
       </c>
-      <c r="K13" s="4">
+      <c r="L13" s="4">
         <v>0.93</v>
       </c>
-      <c r="L13" s="4">
+      <c r="M13" s="4">
         <v>0.08</v>
       </c>
-      <c r="M13" s="4">
-        <v>0</v>
-      </c>
       <c r="N13" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:14" ht="17.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="O13" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" ht="17.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>26</v>
       </c>
@@ -1184,18 +1239,22 @@
         <v>450</v>
       </c>
       <c r="J14" s="6">
+        <f>I14/(1000*F14)</f>
+        <v>1.0843373493975903</v>
+      </c>
+      <c r="K14" s="6">
         <v>100</v>
       </c>
-      <c r="K14" s="6">
+      <c r="L14" s="6">
         <v>0.85</v>
       </c>
-      <c r="L14" s="6">
+      <c r="M14" s="6">
         <v>0.05</v>
       </c>
-      <c r="M14" s="6">
-        <v>0</v>
-      </c>
       <c r="N14" s="6">
+        <v>0</v>
+      </c>
+      <c r="O14" s="6">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
set carbon threshold explicit
</commit_message>
<xml_diff>
--- a/cost_final24.xlsx
+++ b/cost_final24.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\1_UPM_Z\PYsimul\SMR_model1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B09C8DF-2CD6-4C81-9320-E0596127D6AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9809DF6A-E807-424E-8B01-8CB574A3BEF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19090" yWindow="-110" windowWidth="38620" windowHeight="21820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,6 +39,9 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={D0289C43-A833-42EB-B6DD-035525C890A0}</author>
+    <author>tc={056CFB67-E460-445A-AFEB-6CDC8430CD30}</author>
+    <author>tc={24007486-C9D2-4803-9915-B5465F6BE615}</author>
+    <author>tc={04FA7CEE-1B26-40AA-A602-06EB6E5DDC3F}</author>
   </authors>
   <commentList>
     <comment ref="F1" authorId="0" shapeId="0" xr:uid="{D0289C43-A833-42EB-B6DD-035525C890A0}">
@@ -46,7 +49,31 @@
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Relativo al CO2</t>
+    Relativo al CO2: pasar de MWh_th a MWh_e</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="1" shapeId="0" xr:uid="{056CFB67-E460-445A-AFEB-6CDC8430CD30}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Pasar de Energía química en el combustible a MWh_th producido</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="2" shapeId="0" xr:uid="{24007486-C9D2-4803-9915-B5465F6BE615}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Multiplies de previous column by *1/(1000*efficiency): converts gCO2/kWhe to tonCO2/MWh_th. </t>
+      </text>
+    </comment>
+    <comment ref="G14" authorId="3" shapeId="0" xr:uid="{04FA7CEE-1B26-40AA-A602-06EB6E5DDC3F}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Lowest value from IPPC: https://archive.ipcc.ch/publications_and_data/ar4/wg3/en/ch4s4-3-5.html</t>
       </text>
     </comment>
   </commentList>
@@ -54,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>nuclear</t>
   </si>
@@ -138,13 +165,16 @@
   </si>
   <si>
     <t>carbon_intensity1</t>
+  </si>
+  <si>
+    <t>efficiency2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -178,6 +208,12 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -531,14 +567,29 @@
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <threadedComment ref="F1" dT="2025-04-07T12:41:32.37" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{D0289C43-A833-42EB-B6DD-035525C890A0}">
-    <text>Relativo al CO2</text>
+    <text>Relativo al CO2: pasar de MWh_th a MWh_e</text>
+  </threadedComment>
+  <threadedComment ref="G1" dT="2025-05-11T10:34:52.41" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{056CFB67-E460-445A-AFEB-6CDC8430CD30}">
+    <text>Pasar de Energía química en el combustible a MWh_th producido</text>
+  </threadedComment>
+  <threadedComment ref="K1" dT="2025-05-11T10:38:18.81" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{24007486-C9D2-4803-9915-B5465F6BE615}">
+    <text xml:space="preserve">Multiplies de previous column by *1/(1000*efficiency): converts gCO2/kWhe to tonCO2/MWh_th. </text>
+  </threadedComment>
+  <threadedComment ref="G14" dT="2025-05-11T10:49:59.12" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{04FA7CEE-1B26-40AA-A602-06EB6E5DDC3F}">
+    <text>Lowest value from IPPC: https://archive.ipcc.ch/publications_and_data/ar4/wg3/en/ch4s4-3-5.html</text>
+    <extLst>
+      <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
+        <xltc2:checksum>3927874379</xltc2:checksum>
+        <xltc2:hyperlink startIndex="24" length="71" url="https://archive.ipcc.ch/publications_and_data/ar4/wg3/en/ch4s4-3-5.html"/>
+      </x:ext>
+    </extLst>
   </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:P14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.08984375" bestFit="1" customWidth="1"/>
@@ -547,27 +598,28 @@
     <col min="4" max="4" width="6.08984375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.453125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.08984375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.36328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.6328125" customWidth="1"/>
-    <col min="11" max="11" width="9.08984375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.6328125" customWidth="1"/>
-    <col min="14" max="14" width="4.36328125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.08984375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="20" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.453125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="24.26953125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="20" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.08984375" customWidth="1"/>
+    <col min="8" max="8" width="19.08984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.36328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.6328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.6328125" customWidth="1"/>
+    <col min="12" max="12" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.6328125" customWidth="1"/>
+    <col min="15" max="15" width="4.36328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.08984375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="20" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="24.26953125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="20" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="12.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="17" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" ht="17" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>23</v>
       </c>
@@ -587,34 +639,37 @@
         <v>11</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="17" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" ht="17" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -633,36 +688,37 @@
       <c r="F2" s="4">
         <v>0</v>
       </c>
-      <c r="G2" s="4">
+      <c r="G2" s="4"/>
+      <c r="H2" s="4">
         <v>7</v>
       </c>
-      <c r="H2" s="4">
+      <c r="I2" s="4">
         <v>9.33</v>
       </c>
-      <c r="I2" s="4">
-        <v>0</v>
-      </c>
       <c r="J2" s="4">
-        <f>0</f>
         <v>0</v>
       </c>
       <c r="K2" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="L2" s="4">
         <v>1000</v>
       </c>
-      <c r="L2" s="4">
+      <c r="M2" s="4">
         <v>0.85</v>
       </c>
-      <c r="M2" s="4">
+      <c r="N2" s="4">
         <v>0.05</v>
       </c>
-      <c r="N2" s="4">
-        <v>0</v>
-      </c>
       <c r="O2" s="4">
         <v>0</v>
       </c>
+      <c r="P2" s="4">
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:15" ht="17" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" ht="17" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -681,36 +737,37 @@
       <c r="F3" s="4">
         <v>0</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3" s="4"/>
+      <c r="H3" s="4">
         <v>2</v>
       </c>
-      <c r="H3" s="4">
+      <c r="I3" s="4">
         <v>9.33</v>
       </c>
-      <c r="I3" s="4">
-        <v>0</v>
-      </c>
       <c r="J3" s="4">
-        <f>0</f>
         <v>0</v>
       </c>
       <c r="K3" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="L3" s="4">
         <v>1000</v>
       </c>
-      <c r="L3" s="4">
+      <c r="M3" s="4">
         <v>0.85</v>
       </c>
-      <c r="M3" s="4">
+      <c r="N3" s="4">
         <v>0.05</v>
       </c>
-      <c r="N3" s="4">
-        <v>0</v>
-      </c>
       <c r="O3" s="4">
         <v>0</v>
       </c>
+      <c r="P3" s="4">
+        <v>0</v>
+      </c>
     </row>
-    <row r="4" spans="1:15" ht="17" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" ht="17" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -729,36 +786,37 @@
       <c r="F4" s="4">
         <v>0</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="4"/>
+      <c r="H4" s="4">
         <v>1</v>
       </c>
-      <c r="H4" s="4">
-        <v>0</v>
-      </c>
       <c r="I4" s="4">
         <v>0</v>
       </c>
       <c r="J4" s="4">
-        <f>0</f>
         <v>0</v>
       </c>
       <c r="K4" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="L4" s="4">
         <v>50</v>
       </c>
-      <c r="L4" s="4">
+      <c r="M4" s="4">
         <v>0.3</v>
       </c>
-      <c r="M4" s="4">
+      <c r="N4" s="4">
         <v>0.05</v>
       </c>
-      <c r="N4" s="4">
-        <v>0</v>
-      </c>
       <c r="O4" s="4">
         <v>0</v>
       </c>
+      <c r="P4" s="4">
+        <v>0</v>
+      </c>
     </row>
-    <row r="5" spans="1:15" ht="17" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" ht="17" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -777,36 +835,37 @@
       <c r="F5" s="4">
         <v>0</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="4"/>
+      <c r="H5" s="4">
         <v>1</v>
       </c>
-      <c r="H5" s="4">
-        <v>0</v>
-      </c>
       <c r="I5" s="4">
         <v>0</v>
       </c>
       <c r="J5" s="4">
-        <f>0</f>
         <v>0</v>
       </c>
       <c r="K5" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="L5" s="4">
         <v>50</v>
       </c>
-      <c r="L5" s="4">
+      <c r="M5" s="4">
         <v>0.2</v>
       </c>
-      <c r="M5" s="4">
+      <c r="N5" s="4">
         <v>0.05</v>
       </c>
-      <c r="N5" s="4">
-        <v>0</v>
-      </c>
       <c r="O5" s="4">
         <v>0</v>
       </c>
+      <c r="P5" s="4">
+        <v>0</v>
+      </c>
     </row>
-    <row r="6" spans="1:15" ht="17" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" ht="17" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -825,37 +884,38 @@
       <c r="F6" s="4">
         <v>0.59</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="4"/>
+      <c r="H6" s="4">
         <v>2</v>
       </c>
-      <c r="H6" s="4">
+      <c r="I6" s="4">
         <f>50</f>
         <v>50</v>
       </c>
-      <c r="I6" s="4">
+      <c r="J6" s="4">
         <v>450</v>
       </c>
-      <c r="J6" s="4">
-        <f>0</f>
-        <v>0</v>
-      </c>
       <c r="K6" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="L6" s="4">
         <v>500</v>
       </c>
-      <c r="L6" s="4">
+      <c r="M6" s="4">
         <v>0.85</v>
       </c>
-      <c r="M6" s="4">
+      <c r="N6" s="4">
         <v>0.05</v>
       </c>
-      <c r="N6" s="4">
-        <v>0</v>
-      </c>
       <c r="O6" s="4">
         <v>0</v>
       </c>
+      <c r="P6" s="4">
+        <v>0</v>
+      </c>
     </row>
-    <row r="7" spans="1:15" ht="17" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" ht="17" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -874,36 +934,37 @@
       <c r="F7" s="4">
         <v>0.45</v>
       </c>
-      <c r="G7" s="4">
+      <c r="G7" s="4"/>
+      <c r="H7" s="4">
         <v>4</v>
       </c>
-      <c r="H7" s="4">
+      <c r="I7" s="4">
         <v>30</v>
       </c>
-      <c r="I7" s="4">
+      <c r="J7" s="4">
         <v>850</v>
       </c>
-      <c r="J7" s="4">
-        <f>0</f>
-        <v>0</v>
-      </c>
       <c r="K7" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="L7" s="4">
         <v>500</v>
       </c>
-      <c r="L7" s="4">
+      <c r="M7" s="4">
         <v>0.85</v>
       </c>
-      <c r="M7" s="4">
+      <c r="N7" s="4">
         <v>0.05</v>
       </c>
-      <c r="N7" s="4">
-        <v>0</v>
-      </c>
       <c r="O7" s="4">
         <v>0</v>
       </c>
+      <c r="P7" s="4">
+        <v>0</v>
+      </c>
     </row>
-    <row r="8" spans="1:15" ht="17" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" ht="17" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -922,36 +983,37 @@
       <c r="F8" s="4">
         <v>0</v>
       </c>
-      <c r="G8" s="4">
+      <c r="G8" s="4"/>
+      <c r="H8" s="4">
         <v>1</v>
       </c>
-      <c r="H8" s="4">
-        <v>0</v>
-      </c>
       <c r="I8" s="4">
         <v>0</v>
       </c>
       <c r="J8" s="4">
-        <f>0</f>
         <v>0</v>
       </c>
       <c r="K8" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="L8" s="4">
         <v>100</v>
       </c>
-      <c r="L8" s="4">
+      <c r="M8" s="4">
         <v>0.5</v>
       </c>
-      <c r="M8" s="4">
+      <c r="N8" s="4">
         <v>0.05</v>
       </c>
-      <c r="N8" s="4">
-        <v>0</v>
-      </c>
       <c r="O8" s="4">
         <v>0</v>
       </c>
+      <c r="P8" s="4">
+        <v>0</v>
+      </c>
     </row>
-    <row r="9" spans="1:15" ht="17" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" ht="17" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -970,36 +1032,37 @@
       <c r="F9" s="4">
         <v>0</v>
       </c>
-      <c r="G9" s="4">
+      <c r="G9" s="4"/>
+      <c r="H9" s="4">
         <v>6</v>
       </c>
-      <c r="H9" s="4">
-        <v>0</v>
-      </c>
       <c r="I9" s="4">
         <v>0</v>
       </c>
       <c r="J9" s="4">
-        <f>0</f>
         <v>0</v>
       </c>
       <c r="K9" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="L9" s="4">
         <v>500</v>
       </c>
-      <c r="L9" s="4">
+      <c r="M9" s="4">
         <v>0.2</v>
       </c>
-      <c r="M9" s="4">
+      <c r="N9" s="4">
         <v>0.05</v>
       </c>
-      <c r="N9" s="4">
-        <v>0</v>
-      </c>
       <c r="O9" s="4">
         <v>0</v>
       </c>
+      <c r="P9" s="4">
+        <v>0</v>
+      </c>
     </row>
-    <row r="10" spans="1:15" ht="17" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" ht="17" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -1018,37 +1081,38 @@
       <c r="F10" s="4">
         <v>0</v>
       </c>
-      <c r="G10" s="4">
+      <c r="G10" s="4"/>
+      <c r="H10" s="4">
         <v>6</v>
       </c>
-      <c r="H10" s="4">
-        <v>0</v>
-      </c>
       <c r="I10" s="4">
         <v>0</v>
       </c>
       <c r="J10" s="4">
-        <f>0</f>
         <v>0</v>
       </c>
       <c r="K10" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="L10" s="4">
         <v>5</v>
       </c>
-      <c r="L10" s="4">
+      <c r="M10" s="4">
         <f>0.6</f>
         <v>0.6</v>
       </c>
-      <c r="M10" s="4">
+      <c r="N10" s="4">
         <v>0.05</v>
       </c>
-      <c r="N10" s="4">
-        <v>0</v>
-      </c>
       <c r="O10" s="4">
         <v>0</v>
       </c>
+      <c r="P10" s="4">
+        <v>0</v>
+      </c>
     </row>
-    <row r="11" spans="1:15" ht="17" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" ht="17" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -1067,36 +1131,37 @@
       <c r="F11" s="4">
         <v>0</v>
       </c>
-      <c r="G11" s="4">
+      <c r="G11" s="4"/>
+      <c r="H11" s="4">
         <v>6</v>
       </c>
-      <c r="H11" s="4">
-        <v>0</v>
-      </c>
       <c r="I11" s="4">
         <v>0</v>
       </c>
       <c r="J11" s="4">
-        <f>0</f>
         <v>0</v>
       </c>
       <c r="K11" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="L11" s="4">
         <v>50</v>
       </c>
-      <c r="L11" s="4">
+      <c r="M11" s="4">
         <v>0.2</v>
       </c>
-      <c r="M11" s="4">
+      <c r="N11" s="4">
         <v>0.05</v>
       </c>
-      <c r="N11" s="4">
-        <v>0</v>
-      </c>
       <c r="O11" s="4">
         <v>0</v>
       </c>
+      <c r="P11" s="4">
+        <v>0</v>
+      </c>
     </row>
-    <row r="12" spans="1:15" ht="17" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" ht="17" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>24</v>
       </c>
@@ -1120,14 +1185,11 @@
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12" s="4"/>
+      <c r="H12" s="4">
         <f>1</f>
         <v>1</v>
       </c>
-      <c r="H12" s="4">
-        <f>0</f>
-        <v>0</v>
-      </c>
       <c r="I12" s="4">
         <f>0</f>
         <v>0</v>
@@ -1137,27 +1199,31 @@
         <v>0</v>
       </c>
       <c r="K12" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="L12" s="4">
         <f>50</f>
         <v>50</v>
       </c>
-      <c r="L12" s="4">
+      <c r="M12" s="4">
         <f>0.4</f>
         <v>0.4</v>
       </c>
-      <c r="M12" s="4">
+      <c r="N12" s="4">
         <f>0.05</f>
         <v>0.05</v>
       </c>
-      <c r="N12" s="4">
-        <f>0</f>
-        <v>0</v>
-      </c>
       <c r="O12" s="4">
         <f>0</f>
         <v>0</v>
       </c>
+      <c r="P12" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="13" spans="1:15" ht="17.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:16" ht="17.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>25</v>
       </c>
@@ -1176,37 +1242,38 @@
       <c r="F13" s="4">
         <v>0</v>
       </c>
-      <c r="G13" s="4">
+      <c r="G13" s="4"/>
+      <c r="H13" s="4">
         <v>7</v>
       </c>
-      <c r="H13" s="4">
+      <c r="I13" s="4">
         <f>12</f>
         <v>12</v>
       </c>
-      <c r="I13" s="4">
-        <v>0</v>
-      </c>
       <c r="J13" s="4">
-        <f>0</f>
         <v>0</v>
       </c>
       <c r="K13" s="4">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="L13" s="4">
         <v>300</v>
       </c>
-      <c r="L13" s="4">
+      <c r="M13" s="4">
         <v>0.93</v>
       </c>
-      <c r="M13" s="4">
+      <c r="N13" s="4">
         <v>0.08</v>
       </c>
-      <c r="N13" s="4">
-        <v>0</v>
-      </c>
       <c r="O13" s="4">
         <v>0</v>
       </c>
+      <c r="P13" s="4">
+        <v>0</v>
+      </c>
     </row>
-    <row r="14" spans="1:15" ht="17.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:16" ht="17.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>26</v>
       </c>
@@ -1227,34 +1294,37 @@
         <v>0.41499999999999998</v>
       </c>
       <c r="G14" s="6">
+        <v>0.65</v>
+      </c>
+      <c r="H14" s="6">
         <f>2</f>
         <v>2</v>
       </c>
-      <c r="H14" s="6">
+      <c r="I14" s="6">
         <f>50</f>
         <v>50</v>
       </c>
-      <c r="I14" s="6">
+      <c r="J14" s="6">
         <f>450</f>
         <v>450</v>
       </c>
-      <c r="J14" s="6">
-        <f>I14/(1000*F14)</f>
+      <c r="K14" s="6">
+        <f>J14/(1000*F14)</f>
         <v>1.0843373493975903</v>
       </c>
-      <c r="K14" s="6">
+      <c r="L14" s="6">
         <v>100</v>
       </c>
-      <c r="L14" s="6">
+      <c r="M14" s="6">
         <v>0.85</v>
       </c>
-      <c r="M14" s="6">
+      <c r="N14" s="6">
         <v>0.05</v>
       </c>
-      <c r="N14" s="6">
-        <v>0</v>
-      </c>
       <c r="O14" s="6">
+        <v>0</v>
+      </c>
+      <c r="P14" s="6">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
set SMR efficiencies 21 may
</commit_message>
<xml_diff>
--- a/cost_final24.xlsx
+++ b/cost_final24.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\1_UPM_Z\PYsimul\SMR_model1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB3133A3-C443-4958-A6E7-C8A972419F9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB24634A-9C65-4682-814F-77A86B505009}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1560" windowWidth="18910" windowHeight="5030" tabRatio="589" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="23870" yWindow="4280" windowWidth="18910" windowHeight="5480" tabRatio="589" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,11 +38,16 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
+    <author>tc={1DB93E16-5C30-4FDF-9F73-7207FAFB8D18}</author>
+    <author>tc={FCDF6289-C652-4F2A-BE00-A98F71E98A8D}</author>
+    <author>tc={2C80B9E4-7A4C-4355-A557-A800B1A388E2}</author>
     <author>tc={D0289C43-A833-42EB-B6DD-035525C890A0}</author>
     <author>tc={5868225E-6AB4-4960-B0FA-4BF43D4E082F}</author>
     <author>tc={056CFB67-E460-445A-AFEB-6CDC8430CD30}</author>
+    <author>tc={71DADE9C-2171-452B-BABC-21FC760CB8F9}</author>
     <author>tc={A207D967-D633-419B-99F5-A6CB5395A0E2}</author>
     <author>tc={24007486-C9D2-4803-9915-B5465F6BE615}</author>
+    <author>tc={584A61F6-491E-403C-902B-F3836B986624}</author>
     <author>tc={446071B6-973B-49CC-AB09-55799D74CE52}</author>
     <author>tc={EE4B947D-6F9F-4F19-B505-48EFDEDE0B04}</author>
     <author>tc={BE7568EE-7B2D-4E95-BD63-155DA3607F75}</author>
@@ -50,7 +55,31 @@
     <author>tc={E7CAF854-C30D-4E56-8EAC-6E2FD928681F}</author>
   </authors>
   <commentList>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{D0289C43-A833-42EB-B6DD-035525C890A0}">
+    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{1DB93E16-5C30-4FDF-9F73-7207FAFB8D18}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    USD/KWe</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="1" shapeId="0" xr:uid="{FCDF6289-C652-4F2A-BE00-A98F71E98A8D}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    USD/kWe-yr</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="2" shapeId="0" xr:uid="{2C80B9E4-7A4C-4355-A557-A800B1A388E2}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    USD/MWh</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="3" shapeId="0" xr:uid="{D0289C43-A833-42EB-B6DD-035525C890A0}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -58,7 +87,7 @@
     Rendimiento total de cogeneración (Relativo al CO2): pasar de energía química en el combustible a MWh_e/th (con la fórmula que permite comparar entre generadores CHP y single Power o single Heat).</t>
       </text>
     </comment>
-    <comment ref="G1" authorId="1" shapeId="0" xr:uid="{5868225E-6AB4-4960-B0FA-4BF43D4E082F}">
+    <comment ref="G1" authorId="4" shapeId="0" xr:uid="{5868225E-6AB4-4960-B0FA-4BF43D4E082F}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -66,7 +95,7 @@
     Fracción que pasa de Energía química en el combustible a MWh_e producido con cogeneración</t>
       </text>
     </comment>
-    <comment ref="H1" authorId="2" shapeId="0" xr:uid="{056CFB67-E460-445A-AFEB-6CDC8430CD30}">
+    <comment ref="H1" authorId="5" shapeId="0" xr:uid="{056CFB67-E460-445A-AFEB-6CDC8430CD30}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -74,7 +103,15 @@
     Fracción que pasa de Energía química en el combustible a MWh_th producido con cogeneración</t>
       </text>
     </comment>
-    <comment ref="K1" authorId="3" shapeId="0" xr:uid="{A207D967-D633-419B-99F5-A6CB5395A0E2}">
+    <comment ref="J1" authorId="6" shapeId="0" xr:uid="{71DADE9C-2171-452B-BABC-21FC760CB8F9}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    USD/MWh</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="7" shapeId="0" xr:uid="{A207D967-D633-419B-99F5-A6CB5395A0E2}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -82,7 +119,7 @@
     [tCO2/MWh_fuel] Gas PyPSA stoichometric </t>
       </text>
     </comment>
-    <comment ref="L1" authorId="4" shapeId="0" xr:uid="{24007486-C9D2-4803-9915-B5465F6BE615}">
+    <comment ref="L1" authorId="8" shapeId="0" xr:uid="{24007486-C9D2-4803-9915-B5465F6BE615}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -90,7 +127,15 @@
     Multiplies de previous column by *1/CHP_efficiency: converts to obtain tCO2/MWh_output </t>
       </text>
     </comment>
-    <comment ref="Q1" authorId="5" shapeId="0" xr:uid="{446071B6-973B-49CC-AB09-55799D74CE52}">
+    <comment ref="M1" authorId="9" shapeId="0" xr:uid="{584A61F6-491E-403C-902B-F3836B986624}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    MW</t>
+      </text>
+    </comment>
+    <comment ref="Q1" authorId="10" shapeId="0" xr:uid="{446071B6-973B-49CC-AB09-55799D74CE52}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -98,7 +143,7 @@
     USD/tCO2</t>
       </text>
     </comment>
-    <comment ref="A6" authorId="6" shapeId="0" xr:uid="{EE4B947D-6F9F-4F19-B505-48EFDEDE0B04}">
+    <comment ref="A6" authorId="11" shapeId="0" xr:uid="{EE4B947D-6F9F-4F19-B505-48EFDEDE0B04}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -106,7 +151,7 @@
     PyPSA 04 Gas turbine, simple cycle-back pressure L (in 2015 USD currency)</t>
       </text>
     </comment>
-    <comment ref="F6" authorId="7" shapeId="0" xr:uid="{BE7568EE-7B2D-4E95-BD63-155DA3607F75}">
+    <comment ref="F6" authorId="12" shapeId="0" xr:uid="{BE7568EE-7B2D-4E95-BD63-155DA3607F75}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -114,7 +159,7 @@
     TFG calculations (PyPSA, DEA, EPA)</t>
       </text>
     </comment>
-    <comment ref="H6" authorId="8" shapeId="0" xr:uid="{04FA7CEE-1B26-40AA-A602-06EB6E5DDC3F}">
+    <comment ref="H6" authorId="13" shapeId="0" xr:uid="{04FA7CEE-1B26-40AA-A602-06EB6E5DDC3F}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -122,7 +167,7 @@
     Values range from IPPC: https://archive.ipcc.ch/publications_and_data/ar4/wg3/en/ch4s4-3-5.html</t>
       </text>
     </comment>
-    <comment ref="I6" authorId="9" shapeId="0" xr:uid="{E7CAF854-C30D-4E56-8EAC-6E2FD928681F}">
+    <comment ref="I6" authorId="14" shapeId="0" xr:uid="{E7CAF854-C30D-4E56-8EAC-6E2FD928681F}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -584,6 +629,15 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="B1" dT="2025-05-21T18:41:38.51" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{1DB93E16-5C30-4FDF-9F73-7207FAFB8D18}">
+    <text>USD/KWe</text>
+  </threadedComment>
+  <threadedComment ref="C1" dT="2025-05-21T19:11:31.13" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{FCDF6289-C652-4F2A-BE00-A98F71E98A8D}">
+    <text>USD/kWe-yr</text>
+  </threadedComment>
+  <threadedComment ref="D1" dT="2025-05-21T19:11:04.15" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{2C80B9E4-7A4C-4355-A557-A800B1A388E2}">
+    <text>USD/MWh</text>
+  </threadedComment>
   <threadedComment ref="F1" dT="2025-04-07T12:41:32.37" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{D0289C43-A833-42EB-B6DD-035525C890A0}">
     <text>Rendimiento total de cogeneración (Relativo al CO2): pasar de energía química en el combustible a MWh_e/th (con la fórmula que permite comparar entre generadores CHP y single Power o single Heat).</text>
   </threadedComment>
@@ -593,11 +647,17 @@
   <threadedComment ref="H1" dT="2025-05-11T10:34:52.41" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{056CFB67-E460-445A-AFEB-6CDC8430CD30}">
     <text>Fracción que pasa de Energía química en el combustible a MWh_th producido con cogeneración</text>
   </threadedComment>
+  <threadedComment ref="J1" dT="2025-05-21T19:12:06.25" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{71DADE9C-2171-452B-BABC-21FC760CB8F9}">
+    <text>USD/MWh</text>
+  </threadedComment>
   <threadedComment ref="K1" dT="2025-05-15T07:48:40.60" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{A207D967-D633-419B-99F5-A6CB5395A0E2}">
     <text xml:space="preserve">[tCO2/MWh_fuel] Gas PyPSA stoichometric </text>
   </threadedComment>
   <threadedComment ref="L1" dT="2025-05-11T10:38:18.81" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{24007486-C9D2-4803-9915-B5465F6BE615}">
     <text xml:space="preserve">Multiplies de previous column by *1/CHP_efficiency: converts to obtain tCO2/MWh_output </text>
+  </threadedComment>
+  <threadedComment ref="M1" dT="2025-05-21T19:12:19.98" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{584A61F6-491E-403C-902B-F3836B986624}">
+    <text>MW</text>
   </threadedComment>
   <threadedComment ref="Q1" dT="2025-05-17T21:24:54.42" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{446071B6-973B-49CC-AB09-55799D74CE52}">
     <text>USD/tCO2</text>
@@ -961,8 +1021,8 @@
       <c r="N6" s="5">
         <v>0.85</v>
       </c>
-      <c r="O6" s="5">
-        <v>0.05</v>
+      <c r="O6" s="4">
+        <v>0.08</v>
       </c>
       <c r="P6" s="5">
         <v>0</v>

</xml_diff>

<commit_message>
set heatmap and implicit method
</commit_message>
<xml_diff>
--- a/cost_final24.xlsx
+++ b/cost_final24.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\1_UPM_Z\PYsimul\SMR_model1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB24634A-9C65-4682-814F-77A86B505009}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{140BEE4D-5650-4A12-9061-C2E17BA4C4A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23870" yWindow="4280" windowWidth="18910" windowHeight="5480" tabRatio="589" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="640" windowWidth="18910" windowHeight="6780" tabRatio="589" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Set Sensitivity Gas_fuel cost 25 May
</commit_message>
<xml_diff>
--- a/cost_final24.xlsx
+++ b/cost_final24.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\1_UPM_Z\PYsimul\SMR_model1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{140BEE4D-5650-4A12-9061-C2E17BA4C4A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{006C8531-0B62-4D5C-8718-9A467A21E5FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="640" windowWidth="18910" windowHeight="6780" tabRatio="589" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="640" windowWidth="18910" windowHeight="6780" tabRatio="589" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -108,7 +108,7 @@
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    USD/MWh</t>
+    USD/MWh (fuel?? Or electric?</t>
       </text>
     </comment>
     <comment ref="K1" authorId="7" shapeId="0" xr:uid="{A207D967-D633-419B-99F5-A6CB5395A0E2}">
@@ -648,7 +648,7 @@
     <text>Fracción que pasa de Energía química en el combustible a MWh_th producido con cogeneración</text>
   </threadedComment>
   <threadedComment ref="J1" dT="2025-05-21T19:12:06.25" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{71DADE9C-2171-452B-BABC-21FC760CB8F9}">
-    <text>USD/MWh</text>
+    <text>USD/MWh (fuel?? Or electric?</text>
   </threadedComment>
   <threadedComment ref="K1" dT="2025-05-15T07:48:40.60" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{A207D967-D633-419B-99F5-A6CB5395A0E2}">
     <text xml:space="preserve">[tCO2/MWh_fuel] Gas PyPSA stoichometric </text>

</xml_diff>

<commit_message>
set new efficiencies 15 june
</commit_message>
<xml_diff>
--- a/cost_final24.xlsx
+++ b/cost_final24.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\1_UPM_Z\PYsimul\SMR_model1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F2DE70A-92E1-4B95-9E9F-D8C4CFBCE0B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF084023-33FE-45EE-80E4-AA37A8FBD2A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="589" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -49,6 +49,8 @@
     <author>tc={24007486-C9D2-4803-9915-B5465F6BE615}</author>
     <author>tc={584A61F6-491E-403C-902B-F3836B986624}</author>
     <author>tc={446071B6-973B-49CC-AB09-55799D74CE52}</author>
+    <author>tc={AA0DC341-BA22-4348-A936-EE63FE69F7AC}</author>
+    <author>tc={26DF2D7D-BF63-41C1-9482-7EAA57DA55BE}</author>
     <author>tc={EE4B947D-6F9F-4F19-B505-48EFDEDE0B04}</author>
     <author>tc={BE7568EE-7B2D-4E95-BD63-155DA3607F75}</author>
     <author>tc={04FA7CEE-1B26-40AA-A602-06EB6E5DDC3F}</author>
@@ -143,7 +145,23 @@
     USD/tCO2</t>
       </text>
     </comment>
-    <comment ref="A6" authorId="11" shapeId="0" xr:uid="{EE4B947D-6F9F-4F19-B505-48EFDEDE0B04}">
+    <comment ref="F5" authorId="11" shapeId="0" xr:uid="{AA0DC341-BA22-4348-A936-EE63FE69F7AC}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    FUE (fuel utilization Energy)</t>
+      </text>
+    </comment>
+    <comment ref="I5" authorId="12" shapeId="0" xr:uid="{26DF2D7D-BF63-41C1-9482-7EAA57DA55BE}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    En NERL no especifica: dice it varies??</t>
+      </text>
+    </comment>
+    <comment ref="A6" authorId="13" shapeId="0" xr:uid="{EE4B947D-6F9F-4F19-B505-48EFDEDE0B04}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -151,7 +169,7 @@
     PyPSA 04 Gas turbine, simple cycle-back pressure L (in 2015 USD currency)</t>
       </text>
     </comment>
-    <comment ref="F6" authorId="12" shapeId="0" xr:uid="{BE7568EE-7B2D-4E95-BD63-155DA3607F75}">
+    <comment ref="F6" authorId="14" shapeId="0" xr:uid="{BE7568EE-7B2D-4E95-BD63-155DA3607F75}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -159,15 +177,18 @@
     TFG calculations (PyPSA, DEA, EPA)</t>
       </text>
     </comment>
-    <comment ref="H6" authorId="13" shapeId="0" xr:uid="{04FA7CEE-1B26-40AA-A602-06EB6E5DDC3F}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Values range from IPPC: https://archive.ipcc.ch/publications_and_data/ar4/wg3/en/ch4s4-3-5.html</t>
-      </text>
-    </comment>
-    <comment ref="I6" authorId="14" shapeId="0" xr:uid="{E7CAF854-C30D-4E56-8EAC-6E2FD928681F}">
+    <comment ref="H6" authorId="15" shapeId="0" xr:uid="{04FA7CEE-1B26-40AA-A602-06EB6E5DDC3F}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Values range from IPPC: https://archive.ipcc.ch/publications_and_data/ar4/wg3/en/ch4s4-3-5.html
+Reply:
+    calculo del ciclo termodinámico con temperatura útil de 400ºC 
+</t>
+      </text>
+    </comment>
+    <comment ref="I6" authorId="16" shapeId="0" xr:uid="{E7CAF854-C30D-4E56-8EAC-6E2FD928681F}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -252,7 +273,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -281,8 +302,14 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -292,6 +319,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF4CCCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEE0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -323,7 +368,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -342,6 +387,16 @@
     </xf>
     <xf numFmtId="2" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -662,6 +717,12 @@
   <threadedComment ref="Q1" dT="2025-05-17T21:24:54.42" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{446071B6-973B-49CC-AB09-55799D74CE52}">
     <text>USD/tCO2</text>
   </threadedComment>
+  <threadedComment ref="F5" dT="2025-06-14T15:28:23.37" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{AA0DC341-BA22-4348-A936-EE63FE69F7AC}">
+    <text>FUE (fuel utilization Energy)</text>
+  </threadedComment>
+  <threadedComment ref="I5" dT="2025-06-13T18:19:25.77" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{26DF2D7D-BF63-41C1-9482-7EAA57DA55BE}">
+    <text>En NERL no especifica: dice it varies??</text>
+  </threadedComment>
   <threadedComment ref="A6" dT="2025-05-15T16:10:48.49" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{EE4B947D-6F9F-4F19-B505-48EFDEDE0B04}">
     <text>PyPSA 04 Gas turbine, simple cycle-back pressure L (in 2015 USD currency)</text>
   </threadedComment>
@@ -676,6 +737,10 @@
         <xltc2:hyperlink startIndex="24" length="71" url="https://archive.ipcc.ch/publications_and_data/ar4/wg3/en/ch4s4-3-5.html"/>
       </x:ext>
     </extLst>
+  </threadedComment>
+  <threadedComment ref="H6" dT="2025-06-13T18:07:59.00" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{B1947E41-DC3B-4F33-BA0E-A243393866D2}" parentId="{04FA7CEE-1B26-40AA-A602-06EB6E5DDC3F}">
+    <text xml:space="preserve">calculo del ciclo termodinámico con temperatura útil de 400ºC 
+</text>
   </threadedComment>
   <threadedComment ref="I6" dT="2025-05-15T16:14:58.23" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{E7CAF854-C30D-4E56-8EAC-6E2FD928681F}">
     <text>From NREL NG combustion Turbine</text>
@@ -690,20 +755,20 @@
   <cols>
     <col min="1" max="1" width="12.08984375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.81640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="6.08984375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.453125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.26953125" customWidth="1"/>
+    <col min="7" max="7" width="11.453125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.08984375" customWidth="1"/>
     <col min="9" max="9" width="19.08984375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.36328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.7265625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="17.6328125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="17.6328125" customWidth="1"/>
     <col min="13" max="13" width="9.08984375" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12.26953125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="8.6328125" customWidth="1"/>
-    <col min="16" max="16" width="4.36328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="4.7265625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="13.08984375" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="20" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="16.453125" bestFit="1" customWidth="1"/>
@@ -937,13 +1002,16 @@
         <v>60</v>
       </c>
       <c r="F5" s="4">
-        <v>0.41499999999999998</v>
-      </c>
-      <c r="G5" s="4"/>
+        <f>0.5868</f>
+        <v>0.58679999999999999</v>
+      </c>
+      <c r="G5" s="4">
+        <v>0.25</v>
+      </c>
       <c r="H5" s="4">
-        <v>0.44</v>
-      </c>
-      <c r="I5" s="4">
+        <v>0.42</v>
+      </c>
+      <c r="I5" s="10">
         <v>7</v>
       </c>
       <c r="J5" s="4">
@@ -958,7 +1026,7 @@
         <v>0</v>
       </c>
       <c r="M5" s="4">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="N5" s="4">
         <v>0.93</v>
@@ -990,14 +1058,14 @@
       <c r="E6" s="5">
         <v>25</v>
       </c>
-      <c r="F6" s="5">
-        <v>0.59770000000000001</v>
+      <c r="F6" s="8">
+        <v>0.47610000000000002</v>
       </c>
       <c r="G6" s="5">
-        <v>0.35120000000000001</v>
-      </c>
-      <c r="H6" s="5">
-        <v>0.33</v>
+        <v>0.30769999999999997</v>
+      </c>
+      <c r="H6" s="9">
+        <v>0.21</v>
       </c>
       <c r="I6" s="5">
         <f>3</f>
@@ -1011,9 +1079,9 @@
         <f>0.198</f>
         <v>0.19800000000000001</v>
       </c>
-      <c r="L6" s="5">
+      <c r="L6" s="7">
         <f>K6/(F6)</f>
-        <v>0.3312698678266689</v>
+        <v>0.41587901701323249</v>
       </c>
       <c r="M6" s="5">
         <v>100</v>

</xml_diff>

<commit_message>
Set accurate efficiencies for Gas and SMR
</commit_message>
<xml_diff>
--- a/cost_final24.xlsx
+++ b/cost_final24.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\1_UPM_Z\PYsimul\SMR_model1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F2DE70A-92E1-4B95-9E9F-D8C4CFBCE0B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CA69C91-A895-4DF2-BD62-EB046CC600B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="589" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -937,11 +937,13 @@
         <v>60</v>
       </c>
       <c r="F5" s="4">
-        <v>0.41499999999999998</v>
-      </c>
-      <c r="G5" s="4"/>
+        <v>0.5</v>
+      </c>
+      <c r="G5" s="4">
+        <v>0.27879999999999999</v>
+      </c>
       <c r="H5" s="4">
-        <v>0.44</v>
+        <v>0.36</v>
       </c>
       <c r="I5" s="4">
         <v>7</v>
@@ -991,13 +993,13 @@
         <v>25</v>
       </c>
       <c r="F6" s="5">
-        <v>0.59770000000000001</v>
+        <v>0.48</v>
       </c>
       <c r="G6" s="5">
-        <v>0.35120000000000001</v>
+        <v>0.35</v>
       </c>
       <c r="H6" s="5">
-        <v>0.33</v>
+        <v>0.21</v>
       </c>
       <c r="I6" s="5">
         <f>3</f>
@@ -1013,7 +1015,7 @@
       </c>
       <c r="L6" s="5">
         <f>K6/(F6)</f>
-        <v>0.3312698678266689</v>
+        <v>0.41250000000000003</v>
       </c>
       <c r="M6" s="5">
         <v>100</v>

</xml_diff>

<commit_message>
set 100 MW capacity for SMR
</commit_message>
<xml_diff>
--- a/cost_final24.xlsx
+++ b/cost_final24.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\1_UPM_Z\PYsimul\SMR_model1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CA69C91-A895-4DF2-BD62-EB046CC600B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7C47F6B-43C1-4998-BE31-BB4DB4E2BC52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="589" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -960,7 +960,7 @@
         <v>0</v>
       </c>
       <c r="M5" s="4">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="N5" s="4">
         <v>0.93</v>

</xml_diff>

<commit_message>
set run time drop
</commit_message>
<xml_diff>
--- a/cost_final24.xlsx
+++ b/cost_final24.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\1_UPM_Z\PYsimul\SMR_model1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04C2E959-D291-4B17-ABCD-BE2FF63D137A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40E06A39-EB0E-480F-B776-63898826B363}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="589" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -145,7 +145,7 @@
     USD/tCO2</t>
       </text>
     </comment>
-    <comment ref="F5" authorId="11" shapeId="0" xr:uid="{AA0DC341-BA22-4348-A936-EE63FE69F7AC}">
+    <comment ref="F3" authorId="11" shapeId="0" xr:uid="{AA0DC341-BA22-4348-A936-EE63FE69F7AC}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -153,7 +153,7 @@
     FUE (fuel utilization Energy)</t>
       </text>
     </comment>
-    <comment ref="I5" authorId="12" shapeId="0" xr:uid="{26DF2D7D-BF63-41C1-9482-7EAA57DA55BE}">
+    <comment ref="I3" authorId="12" shapeId="0" xr:uid="{26DF2D7D-BF63-41C1-9482-7EAA57DA55BE}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -161,7 +161,7 @@
     En NERL no especifica: dice it varies??</t>
       </text>
     </comment>
-    <comment ref="A6" authorId="13" shapeId="0" xr:uid="{EE4B947D-6F9F-4F19-B505-48EFDEDE0B04}">
+    <comment ref="A4" authorId="13" shapeId="0" xr:uid="{EE4B947D-6F9F-4F19-B505-48EFDEDE0B04}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -169,7 +169,7 @@
     PyPSA 04 Gas turbine, simple cycle-back pressure L (in 2015 USD currency)</t>
       </text>
     </comment>
-    <comment ref="F6" authorId="14" shapeId="0" xr:uid="{BE7568EE-7B2D-4E95-BD63-155DA3607F75}">
+    <comment ref="F4" authorId="14" shapeId="0" xr:uid="{BE7568EE-7B2D-4E95-BD63-155DA3607F75}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -177,7 +177,7 @@
     TFG calculations (PyPSA, DEA, EPA)</t>
       </text>
     </comment>
-    <comment ref="H6" authorId="15" shapeId="0" xr:uid="{04FA7CEE-1B26-40AA-A602-06EB6E5DDC3F}">
+    <comment ref="H4" authorId="15" shapeId="0" xr:uid="{04FA7CEE-1B26-40AA-A602-06EB6E5DDC3F}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -188,7 +188,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="I6" authorId="16" shapeId="0" xr:uid="{E7CAF854-C30D-4E56-8EAC-6E2FD928681F}">
+    <comment ref="I4" authorId="16" shapeId="0" xr:uid="{E7CAF854-C30D-4E56-8EAC-6E2FD928681F}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -201,13 +201,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
-  <si>
-    <t>nuclear</t>
-  </si>
-  <si>
-    <t>nuclear_lto</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>CCGT</t>
   </si>
@@ -711,19 +705,19 @@
   <threadedComment ref="Q1" dT="2025-05-17T21:24:54.42" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{446071B6-973B-49CC-AB09-55799D74CE52}">
     <text>USD/tCO2</text>
   </threadedComment>
-  <threadedComment ref="F5" dT="2025-06-14T15:28:23.37" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{AA0DC341-BA22-4348-A936-EE63FE69F7AC}">
+  <threadedComment ref="F3" dT="2025-06-14T15:28:23.37" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{AA0DC341-BA22-4348-A936-EE63FE69F7AC}">
     <text>FUE (fuel utilization Energy)</text>
   </threadedComment>
-  <threadedComment ref="I5" dT="2025-06-13T18:19:25.77" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{26DF2D7D-BF63-41C1-9482-7EAA57DA55BE}">
+  <threadedComment ref="I3" dT="2025-06-13T18:19:25.77" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{26DF2D7D-BF63-41C1-9482-7EAA57DA55BE}">
     <text>En NERL no especifica: dice it varies??</text>
   </threadedComment>
-  <threadedComment ref="A6" dT="2025-05-15T16:10:48.49" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{EE4B947D-6F9F-4F19-B505-48EFDEDE0B04}">
+  <threadedComment ref="A4" dT="2025-05-15T16:10:48.49" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{EE4B947D-6F9F-4F19-B505-48EFDEDE0B04}">
     <text>PyPSA 04 Gas turbine, simple cycle-back pressure L (in 2015 USD currency)</text>
   </threadedComment>
-  <threadedComment ref="F6" dT="2025-05-17T09:37:28.80" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{BE7568EE-7B2D-4E95-BD63-155DA3607F75}">
+  <threadedComment ref="F4" dT="2025-05-17T09:37:28.80" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{BE7568EE-7B2D-4E95-BD63-155DA3607F75}">
     <text>TFG calculations (PyPSA, DEA, EPA)</text>
   </threadedComment>
-  <threadedComment ref="H6" dT="2025-05-11T10:49:59.12" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{04FA7CEE-1B26-40AA-A602-06EB6E5DDC3F}">
+  <threadedComment ref="H4" dT="2025-05-11T10:49:59.12" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{04FA7CEE-1B26-40AA-A602-06EB6E5DDC3F}">
     <text>Values range from IPPC: https://archive.ipcc.ch/publications_and_data/ar4/wg3/en/ch4s4-3-5.html</text>
     <extLst>
       <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
@@ -732,11 +726,11 @@
       </x:ext>
     </extLst>
   </threadedComment>
-  <threadedComment ref="H6" dT="2025-06-13T18:07:59.00" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{B1947E41-DC3B-4F33-BA0E-A243393866D2}" parentId="{04FA7CEE-1B26-40AA-A602-06EB6E5DDC3F}">
+  <threadedComment ref="H4" dT="2025-06-13T18:07:59.00" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{B1947E41-DC3B-4F33-BA0E-A243393866D2}" parentId="{04FA7CEE-1B26-40AA-A602-06EB6E5DDC3F}">
     <text xml:space="preserve">calculo del ciclo termodinámico con temperatura útil de 400ºC 
 </text>
   </threadedComment>
-  <threadedComment ref="I6" dT="2025-05-15T16:14:58.23" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{E7CAF854-C30D-4E56-8EAC-6E2FD928681F}">
+  <threadedComment ref="I4" dT="2025-05-15T16:14:58.23" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{E7CAF854-C30D-4E56-8EAC-6E2FD928681F}">
     <text>From NREL NG combustion Turbine</text>
   </threadedComment>
 </ThreadedComments>
@@ -744,7 +738,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:Q4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.08984375" bestFit="1" customWidth="1"/>
@@ -777,93 +771,94 @@
   <sheetData>
     <row r="1" spans="1:17" ht="17" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="F1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="N1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="2" t="s">
+      <c r="O1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="P1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="N1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>15</v>
-      </c>
     </row>
-    <row r="2" spans="1:17" ht="17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:17" ht="17" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="3">
-        <v>6000</v>
+      <c r="B2" s="4">
+        <v>750</v>
       </c>
       <c r="C2" s="4">
-        <v>100</v>
+        <v>20.167538959821201</v>
       </c>
       <c r="D2" s="4">
-        <v>2</v>
+        <v>1.827</v>
       </c>
       <c r="E2" s="4">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F2" s="4">
-        <v>0</v>
+        <v>0.59</v>
       </c>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J2" s="4">
-        <v>9.33</v>
+        <f>50</f>
+        <v>50</v>
       </c>
       <c r="K2" s="4">
-        <v>0</v>
+        <v>450</v>
       </c>
       <c r="L2" s="4">
         <f>0</f>
         <v>0</v>
       </c>
       <c r="M2" s="4">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="N2" s="4">
         <v>0.85</v>
@@ -878,32 +873,38 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:17" ht="17.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="2" t="s">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="B3" s="3">
-        <v>750</v>
+        <v>9500</v>
       </c>
       <c r="C3" s="4">
-        <v>100</v>
+        <v>216</v>
       </c>
       <c r="D3" s="4">
-        <v>4</v>
+        <v>2.8</v>
       </c>
       <c r="E3" s="4">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="F3" s="4">
-        <v>0</v>
-      </c>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4">
-        <v>2</v>
+        <f>0.5868</f>
+        <v>0.58679999999999999</v>
+      </c>
+      <c r="G3" s="4">
+        <v>0.27879999999999999</v>
+      </c>
+      <c r="H3" s="4">
+        <v>0.21</v>
+      </c>
+      <c r="I3" s="9">
+        <v>7</v>
       </c>
       <c r="J3" s="4">
-        <v>9.33</v>
+        <f>12</f>
+        <v>12</v>
       </c>
       <c r="K3" s="4">
         <v>0</v>
@@ -913,13 +914,13 @@
         <v>0</v>
       </c>
       <c r="M3" s="4">
-        <v>1000</v>
+        <v>100</v>
       </c>
       <c r="N3" s="4">
-        <v>0.85</v>
+        <v>0.93</v>
       </c>
       <c r="O3" s="4">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
       <c r="P3" s="4">
         <v>0</v>
@@ -928,168 +929,61 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:17" ht="17.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="4">
-        <v>750</v>
-      </c>
-      <c r="C4" s="4">
-        <v>20.167538959821201</v>
-      </c>
-      <c r="D4" s="4">
-        <v>1.827</v>
-      </c>
-      <c r="E4" s="4">
-        <v>30</v>
-      </c>
-      <c r="F4" s="4">
-        <v>0.59</v>
-      </c>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4">
-        <v>2</v>
-      </c>
-      <c r="J4" s="4">
+        <v>16</v>
+      </c>
+      <c r="B4" s="5">
+        <f>583.13</f>
+        <v>583.13</v>
+      </c>
+      <c r="C4" s="5">
+        <v>20.63</v>
+      </c>
+      <c r="D4" s="6">
+        <v>5.5</v>
+      </c>
+      <c r="E4" s="5">
+        <v>25</v>
+      </c>
+      <c r="F4" s="10">
+        <v>0.47610000000000002</v>
+      </c>
+      <c r="G4" s="5">
+        <v>0.30769999999999997</v>
+      </c>
+      <c r="H4" s="8">
+        <v>0.21</v>
+      </c>
+      <c r="I4" s="5">
+        <f>3</f>
+        <v>3</v>
+      </c>
+      <c r="J4" s="5">
         <f>50</f>
         <v>50</v>
       </c>
-      <c r="K4" s="4">
-        <v>450</v>
-      </c>
-      <c r="L4" s="4">
-        <f>0</f>
-        <v>0</v>
-      </c>
-      <c r="M4" s="4">
-        <v>500</v>
-      </c>
-      <c r="N4" s="4">
-        <v>0.85</v>
-      </c>
-      <c r="O4" s="4">
-        <v>0.05</v>
-      </c>
-      <c r="P4" s="4">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" ht="17.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="3">
-        <v>9500</v>
-      </c>
-      <c r="C5" s="4">
-        <v>216</v>
-      </c>
-      <c r="D5" s="4">
-        <v>2.8</v>
-      </c>
-      <c r="E5" s="4">
-        <v>60</v>
-      </c>
-      <c r="F5" s="4">
-        <f>0.5868</f>
-        <v>0.58679999999999999</v>
-      </c>
-      <c r="G5" s="4">
-        <v>0.27879999999999999</v>
-      </c>
-      <c r="H5" s="4">
-        <v>0.21</v>
-      </c>
-      <c r="I5" s="9">
-        <v>7</v>
-      </c>
-      <c r="J5" s="4">
-        <f>12</f>
-        <v>12</v>
-      </c>
-      <c r="K5" s="4">
-        <v>0</v>
-      </c>
-      <c r="L5" s="4">
-        <f>0</f>
-        <v>0</v>
-      </c>
-      <c r="M5" s="4">
-        <v>100</v>
-      </c>
-      <c r="N5" s="4">
-        <v>0.93</v>
-      </c>
-      <c r="O5" s="4">
-        <v>0.08</v>
-      </c>
-      <c r="P5" s="4">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" ht="17.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" s="5">
-        <f>583.13</f>
-        <v>583.13</v>
-      </c>
-      <c r="C6" s="5">
-        <v>20.63</v>
-      </c>
-      <c r="D6" s="6">
-        <v>5.5</v>
-      </c>
-      <c r="E6" s="5">
-        <v>25</v>
-      </c>
-      <c r="F6" s="10">
-        <v>0.47610000000000002</v>
-      </c>
-      <c r="G6" s="5">
-        <v>0.30769999999999997</v>
-      </c>
-      <c r="H6" s="8">
-        <v>0.21</v>
-      </c>
-      <c r="I6" s="5">
-        <f>3</f>
-        <v>3</v>
-      </c>
-      <c r="J6" s="5">
-        <f>50</f>
-        <v>50</v>
-      </c>
-      <c r="K6" s="5">
+      <c r="K4" s="5">
         <f>0.198</f>
         <v>0.19800000000000001</v>
       </c>
-      <c r="L6" s="7">
-        <f>K6/(F6)</f>
+      <c r="L4" s="7">
+        <f>K4/(F4)</f>
         <v>0.41587901701323249</v>
       </c>
-      <c r="M6" s="5">
+      <c r="M4" s="5">
         <v>100</v>
       </c>
-      <c r="N6" s="5">
+      <c r="N4" s="5">
         <v>0.85</v>
       </c>
-      <c r="O6" s="4">
+      <c r="O4" s="4">
         <v>0.08</v>
       </c>
-      <c r="P6" s="5">
+      <c r="P4" s="5">
         <v>0</v>
       </c>
-      <c r="Q6" s="5">
+      <c r="Q4" s="5">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
set SIDNE+ legends new
</commit_message>
<xml_diff>
--- a/cost_final24.xlsx
+++ b/cost_final24.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\1_UPM_Z\PYsimul\SMR_model1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40E06A39-EB0E-480F-B776-63898826B363}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF23273F-C81D-4064-BB9E-568A949FD5F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="589" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -55,6 +55,7 @@
     <author>tc={BE7568EE-7B2D-4E95-BD63-155DA3607F75}</author>
     <author>tc={04FA7CEE-1B26-40AA-A602-06EB6E5DDC3F}</author>
     <author>tc={E7CAF854-C30D-4E56-8EAC-6E2FD928681F}</author>
+    <author>tc={ED393121-FA30-41D4-A2D4-B6CBE6D9672B}</author>
   </authors>
   <commentList>
     <comment ref="B1" authorId="0" shapeId="0" xr:uid="{1DB93E16-5C30-4FDF-9F73-7207FAFB8D18}">
@@ -194,6 +195,14 @@
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     From NREL NG combustion Turbine</t>
+      </text>
+    </comment>
+    <comment ref="Q4" authorId="17" shapeId="0" xr:uid="{ED393121-FA30-41D4-A2D4-B6CBE6D9672B}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Se añade en cada código para poder aplicar el método implícito</t>
       </text>
     </comment>
   </commentList>
@@ -267,7 +276,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -295,6 +304,12 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="6">
@@ -733,6 +748,9 @@
   <threadedComment ref="I4" dT="2025-05-15T16:14:58.23" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{E7CAF854-C30D-4E56-8EAC-6E2FD928681F}">
     <text>From NREL NG combustion Turbine</text>
   </threadedComment>
+  <threadedComment ref="Q4" dT="2025-06-18T19:45:29.33" personId="{C4A57D0B-4E4B-4986-94C7-8988CF687508}" id="{ED393121-FA30-41D4-A2D4-B6CBE6D9672B}">
+    <text>Se añade en cada código para poder aplicar el método implícito</text>
+  </threadedComment>
 </ThreadedComments>
 </file>
 

</xml_diff>